<commit_message>
update master barang dan barang masuk
</commit_message>
<xml_diff>
--- a/storage/app/templates/template_master_barang.xlsx
+++ b/storage/app/templates/template_master_barang.xlsx
@@ -424,13 +424,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -454,6 +455,11 @@
           <t>Satuan Default</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Spesifikasi Default</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -476,6 +482,11 @@
           <t>Botol</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Tinta Epson Hitam</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -498,6 +509,7 @@
           <t>Buah</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>